<commit_message>
Update inventory for riyadh - 1785270738530
</commit_message>
<xml_diff>
--- a/stores/riyadh.xlsx
+++ b/stores/riyadh.xlsx
@@ -109,6 +109,53 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr" s="2">
+        <is>
+          <t>9521000999992</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr" s="2">
+        <is>
+          <t>1-2-3</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr" s="2">
+        <is>
+          <t>1785270719804</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr" s="2">
+        <is>
+          <t>1785270719803</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr" s="2">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory for riyadh - 1785296714557
</commit_message>
<xml_diff>
--- a/stores/riyadh.xlsx
+++ b/stores/riyadh.xlsx
@@ -103,11 +103,6 @@
           <t>CreatedAt</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="1">
-        <is>
-          <t>SyncStatus</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
@@ -150,9 +145,46 @@
           <t>1785270719803</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr" s="2">
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr" s="2">
         <is>
-          <t>PENDING</t>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="2">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="2">
+        <is>
+          <t>3-2-1</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr" s="2">
+        <is>
+          <t>1785272145733</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr" s="2">
+        <is>
+          <t>1785272145732</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update inventory for riyadh - 1785298653621
</commit_message>
<xml_diff>
--- a/stores/riyadh.xlsx
+++ b/stores/riyadh.xlsx
@@ -188,6 +188,48 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="2">
+        <is>
+          <t>6970903969381</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="2">
+        <is>
+          <t>3-1-3</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr" s="2">
+        <is>
+          <t>1785298640969</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr" s="2">
+        <is>
+          <t>1785298640968</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>